<commit_message>
added Donor column to templates, examples, and flatteners
</commit_message>
<xml_diff>
--- a/Organization_Template_Alternate_example_data.xlsx
+++ b/Organization_Template_Alternate_example_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\marnold\phpOrganizationsBuilder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99BD5E1-8EE1-4BB6-B12F-16DBDFD3CAF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2FDE41-724D-47BB-B2FD-E93DAD80B50C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29745" yWindow="1140" windowWidth="25050" windowHeight="13140" tabRatio="731" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="285" yWindow="435" windowWidth="21600" windowHeight="11295" tabRatio="731" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use this workbook" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="441">
   <si>
     <t>ORG CODE*</t>
   </si>
@@ -1351,6 +1351,9 @@
   </si>
   <si>
     <t>ACCT-9001</t>
+  </si>
+  <si>
+    <t>Donor (Yes/No)</t>
   </si>
 </sst>
 </file>
@@ -1467,7 +1470,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1511,13 +1514,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2635,31 +2637,31 @@
   <sheetPr>
     <tabColor rgb="FFFFF2CC"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
     <col min="2" max="2" width="25.42578125" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="13"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -2670,36 +2672,42 @@
         <v>39</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="G5" s="12" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="21" t="s">
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="F6" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="G6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2710,16 +2718,19 @@
         <v>44</v>
       </c>
       <c r="D7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" t="s">
         <v>45</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>49</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -2730,16 +2741,19 @@
         <v>44</v>
       </c>
       <c r="D8" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" t="s">
         <v>45</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>52</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -2750,16 +2764,19 @@
         <v>44</v>
       </c>
       <c r="D9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" t="s">
         <v>45</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>55</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -2770,16 +2787,19 @@
         <v>44</v>
       </c>
       <c r="D10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" t="s">
         <v>45</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>58</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>60</v>
       </c>
@@ -2790,13 +2810,16 @@
         <v>62</v>
       </c>
       <c r="D11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" t="s">
         <v>45</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>64</v>
       </c>
@@ -2807,16 +2830,19 @@
         <v>44</v>
       </c>
       <c r="D12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" t="s">
         <v>45</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>66</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>68</v>
       </c>
@@ -2827,10 +2853,13 @@
         <v>62</v>
       </c>
       <c r="D13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>71</v>
       </c>
@@ -2841,16 +2870,19 @@
         <v>44</v>
       </c>
       <c r="D14" t="s">
+        <v>62</v>
+      </c>
+      <c r="E14" t="s">
         <v>45</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>73</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>75</v>
       </c>
@@ -2861,13 +2893,16 @@
         <v>62</v>
       </c>
       <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" t="s">
         <v>45</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>78</v>
       </c>
@@ -2878,16 +2913,19 @@
         <v>44</v>
       </c>
       <c r="D16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" t="s">
         <v>45</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>80</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>81</v>
       </c>
@@ -2898,16 +2936,19 @@
         <v>44</v>
       </c>
       <c r="D17" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17" t="s">
         <v>45</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>84</v>
       </c>
@@ -2918,16 +2959,19 @@
         <v>44</v>
       </c>
       <c r="D18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" t="s">
         <v>45</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>87</v>
       </c>
@@ -2938,13 +2982,16 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" t="s">
         <v>45</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>90</v>
       </c>
@@ -2955,13 +3002,16 @@
         <v>62</v>
       </c>
       <c r="D20" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" t="s">
         <v>45</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>93</v>
       </c>
@@ -2972,16 +3022,19 @@
         <v>44</v>
       </c>
       <c r="D21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" t="s">
         <v>45</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>95</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>96</v>
       </c>
@@ -2992,13 +3045,16 @@
         <v>62</v>
       </c>
       <c r="D22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" t="s">
         <v>45</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>99</v>
       </c>
@@ -3009,16 +3065,19 @@
         <v>44</v>
       </c>
       <c r="D23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" t="s">
         <v>45</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>101</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>102</v>
       </c>
@@ -3029,13 +3088,16 @@
         <v>62</v>
       </c>
       <c r="D24" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" t="s">
         <v>45</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -3046,24 +3108,27 @@
         <v>44</v>
       </c>
       <c r="D25" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" t="s">
         <v>106</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>107</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>74</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:D1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:D1048576" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E1048576" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Active, Inactive, Pending"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6:G1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Access provider,Auction house,Book trade,Consortium,Content provider,Logistics,Material supplier,Membership organization,Private person,Publisher"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3697,31 +3762,31 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" t="s">
         <v>196</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" t="s">
         <v>197</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" t="s">
         <v>198</v>
       </c>
-      <c r="E3" s="21" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" t="s">
         <v>199</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" t="s">
         <v>200</v>
       </c>
     </row>
@@ -3965,31 +4030,31 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" t="s">
         <v>222</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" t="s">
         <v>223</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" t="s">
         <v>224</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" t="s">
         <v>225</v>
       </c>
-      <c r="F3" s="21" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+      <c r="F3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" t="s">
         <v>226</v>
       </c>
     </row>
@@ -4424,40 +4489,40 @@
       </c>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" s="21" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" t="s">
         <v>272</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" t="s">
         <v>273</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" t="s">
         <v>274</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" t="s">
         <v>275</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" t="s">
         <v>276</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" t="s">
         <v>277</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="H3" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="21" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+    <row r="4" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" t="s">
         <v>278</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" t="s">
         <v>279</v>
       </c>
     </row>
@@ -4646,10 +4711,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="21" t="s">
         <v>316</v>
       </c>
-      <c r="G1" s="20"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -4677,43 +4742,43 @@
         <v>269</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" t="s">
         <v>322</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" t="s">
         <v>323</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="19" t="s">
         <v>324</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" t="s">
         <v>325</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" t="s">
         <v>326</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" t="s">
         <v>327</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="H3" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" t="s">
         <v>329</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" t="s">
         <v>330</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" t="s">
         <v>331</v>
       </c>
     </row>

</xml_diff>